<commit_message>
Add worker wages PDF for sharing
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/أجور_العمال.xlsx
+++ b/أجور_العمال.xlsx
@@ -10,7 +10,10 @@
     <sheet name="أجور 08-2026" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="أجور 04-2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'أجور 08-2026'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'أجور 04-2026'!$1:$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -498,7 +501,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2032,7 +2035,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2040,7 +2044,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3667,6 +3671,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>